<commit_message>
Major update. Many diagnostics have been run and can be commented out or deleted later. In broad terms, what have been changed are: Added Scope 1, 2, and 3 calculations + a Fourth graph to visualize these (fig_scope), added a fifth 'total' graph where bottomup calculations are added. 'Transport' disaggregated from 'others' due to the significane in the results (this is also why so many diagnostics were necessary; to make sure that the significance of 'transport' was not caused by calculation or modelling mistakes). Added bottomup data by scaling Dutch values (using scaling as a method to calculate emissions in all 5 emission categories was done to avoid  inconsistencies between ecoinvent methodologies)
</commit_message>
<xml_diff>
--- a/output/Table1.xlsx
+++ b/output/Table1.xlsx
@@ -441,22 +441,22 @@
         <v>6</v>
       </c>
       <c r="B2">
-        <v>19792.54129835656</v>
+        <v>4667.930812962716</v>
       </c>
       <c r="C2">
-        <v>15066.47555447738</v>
+        <v>2542.230129466179</v>
       </c>
       <c r="D2">
-        <v>621.6720529563064</v>
+        <v>45.33592242512116</v>
       </c>
       <c r="E2">
-        <v>30290.74036012588</v>
+        <v>2669.231027940203</v>
       </c>
       <c r="F2">
-        <v>5701.982570874461</v>
+        <v>815.1555705483208</v>
       </c>
       <c r="G2">
-        <v>92528.019626516</v>
+        <v>24822.19302474687</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -464,22 +464,22 @@
         <v>7</v>
       </c>
       <c r="B3">
-        <v>11692.00206736152</v>
+        <v>3147.102279461976</v>
       </c>
       <c r="C3">
-        <v>7093.838029203962</v>
+        <v>1250.784083373463</v>
       </c>
       <c r="D3">
-        <v>302.4603624540867</v>
+        <v>25.87712577424498</v>
       </c>
       <c r="E3">
-        <v>16324.85947714854</v>
+        <v>1799.609715926473</v>
       </c>
       <c r="F3">
-        <v>3109.280991178463</v>
+        <v>536.5781148051582</v>
       </c>
       <c r="G3">
-        <v>86096</v>
+        <v>22186.57530201342</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -487,22 +487,22 @@
         <v>8</v>
       </c>
       <c r="B4">
-        <v>6131.186826176758</v>
+        <v>755.74725607912</v>
       </c>
       <c r="C4">
-        <v>7385.415563697593</v>
+        <v>1132.102781893308</v>
       </c>
       <c r="D4">
-        <v>309.6276001236665</v>
+        <v>17.12134480743643</v>
       </c>
       <c r="E4">
-        <v>13515.18985424745</v>
+        <v>754.5313705773699</v>
       </c>
       <c r="F4">
-        <v>2312.637594047707</v>
+        <v>221.2743803567267</v>
       </c>
       <c r="G4">
-        <v>3792.926263700311</v>
+        <v>1734.622069918767</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -510,22 +510,22 @@
         <v>9</v>
       </c>
       <c r="B5">
-        <v>946.1838048182954</v>
+        <v>180.9222774216217</v>
       </c>
       <c r="C5">
-        <v>545.0428615758075</v>
+        <v>134.6903641994151</v>
       </c>
       <c r="D5">
-        <v>9.291590378553938</v>
+        <v>2.166151843439692</v>
       </c>
       <c r="E5">
-        <v>447.9448287298518</v>
+        <v>113.485041436354</v>
       </c>
       <c r="F5">
-        <v>280.063985648286</v>
+        <v>57.30307538643692</v>
       </c>
       <c r="G5">
-        <v>2639.093362815687</v>
+        <v>900.9956528146802</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -533,7 +533,7 @@
         <v>10</v>
       </c>
       <c r="B6">
-        <v>14.2</v>
+        <v>9.513999999999999</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -556,7 +556,7 @@
         <v>11</v>
       </c>
       <c r="B7">
-        <v>76.90000000000001</v>
+        <v>34.605</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -579,16 +579,16 @@
         <v>12</v>
       </c>
       <c r="B8">
-        <v>932.0685999999999</v>
+        <v>540.04</v>
       </c>
       <c r="C8">
-        <v>42.17910000000001</v>
+        <v>24.6529</v>
       </c>
       <c r="D8">
-        <v>0.2925</v>
+        <v>0.1713</v>
       </c>
       <c r="E8">
-        <v>2.7462</v>
+        <v>1.6049</v>
       </c>
       <c r="F8">
         <v>0</v>

</xml_diff>